<commit_message>
Mise à jour scripts Romain + ajout PM AS Indus
</commit_message>
<xml_diff>
--- a/03_intermediary_data/Table_correspondance.xlsx
+++ b/03_intermediary_data/Table_correspondance.xlsx
@@ -2919,8 +2919,8 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E0B707973A0EDF4D8C0132D38830BF56" ma:contentTypeVersion="3" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="633c736c1f52b59bab6ff2ec826f3b7e">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4222387a-a7c4-4a56-bf01-5dca1ac56634" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="a8c24be4bccf061f1609b4dbaef8d8d2" ns2:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100E0B707973A0EDF4D8C0132D38830BF56" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6fab73de96728382b95836a8b817e49f">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="4222387a-a7c4-4a56-bf01-5dca1ac56634" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="2d5a3db95c4c940e29da1a6f70bc1044" ns2:_="">
     <xsd:import namespace="4222387a-a7c4-4a56-bf01-5dca1ac56634"/>
     <xsd:element name="properties">
       <xsd:complexType>
@@ -2966,8 +2966,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Type de contenu"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titre"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -3072,21 +3072,7 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21C86FAE-DA48-488B-A9BC-622ABC856A92}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="4222387a-a7c4-4a56-bf01-5dca1ac56634"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{49494ED9-69F9-4069-9BE4-58956FA79713}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>